<commit_message>
feat: Tratar relatorio BRF
</commit_message>
<xml_diff>
--- a/ModelorelatorioBRF.xlsx
+++ b/ModelorelatorioBRF.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mfs\usuarios\dionathan.silva\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\magna_gestao_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9820FAA-0B97-4B16-BD3B-71AC9C57372B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F323A06-BCE5-4889-BD42-3553445AD795}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CCE919F5-458D-4DD3-A4E6-55BE21981BE5}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="213">
   <si>
     <t>Transportador</t>
   </si>
@@ -1015,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A3233E8-725F-4E69-ABE4-C814CF00BAEC}">
-  <dimension ref="A1:AD39"/>
+  <dimension ref="A1:AD37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -2450,16 +2450,16 @@
         <v>34</v>
       </c>
       <c r="G16" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="H16" t="s">
-        <v>40</v>
+        <v>126</v>
       </c>
       <c r="I16" t="s">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="J16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K16">
         <v>12650</v>
@@ -2471,7 +2471,7 @@
         <v>417.72</v>
       </c>
       <c r="N16" t="s">
-        <v>40</v>
+        <v>127</v>
       </c>
       <c r="O16" t="s">
         <v>40</v>
@@ -2483,7 +2483,7 @@
         <v>1</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S16" t="s">
         <v>59</v>
@@ -2530,40 +2530,40 @@
         <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D17" t="s">
-        <v>40</v>
+        <v>129</v>
       </c>
       <c r="E17">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="F17" t="s">
         <v>34</v>
       </c>
       <c r="G17" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="H17" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="I17" t="s">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="J17" t="s">
         <v>38</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>13400</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>93.78</v>
       </c>
       <c r="M17">
-        <v>0</v>
+        <v>645.67999999999995</v>
       </c>
       <c r="N17" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="O17" t="s">
         <v>40</v>
@@ -2572,19 +2572,19 @@
         <v>41</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="T17" t="s">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="U17" t="s">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="V17" t="s">
         <v>45</v>
@@ -2599,7 +2599,7 @@
         <v>48</v>
       </c>
       <c r="Z17" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="AA17" t="s">
         <v>50</v>
@@ -2611,7 +2611,7 @@
         <v>52</v>
       </c>
       <c r="AD17" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.25">
@@ -2622,40 +2622,40 @@
         <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D18" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E18">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="F18" t="s">
         <v>34</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H18" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="I18" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="J18" t="s">
         <v>38</v>
       </c>
       <c r="K18">
-        <v>13400</v>
+        <v>12390</v>
       </c>
       <c r="L18">
-        <v>93.78</v>
+        <v>73.81</v>
       </c>
       <c r="M18">
-        <v>645.67999999999995</v>
+        <v>519.48</v>
       </c>
       <c r="N18" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="O18" t="s">
         <v>40</v>
@@ -2714,10 +2714,10 @@
         <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D19" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E19">
         <v>46203</v>
@@ -2726,28 +2726,28 @@
         <v>34</v>
       </c>
       <c r="G19" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H19" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="I19" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="J19" t="s">
         <v>38</v>
       </c>
       <c r="K19">
-        <v>12390</v>
+        <v>13700</v>
       </c>
       <c r="L19">
-        <v>73.81</v>
+        <v>49.7</v>
       </c>
       <c r="M19">
-        <v>519.48</v>
+        <v>470.89</v>
       </c>
       <c r="N19" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="O19" t="s">
         <v>40</v>
@@ -2762,7 +2762,7 @@
         <v>1</v>
       </c>
       <c r="S19" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="T19" t="s">
         <v>43</v>
@@ -2795,7 +2795,7 @@
         <v>52</v>
       </c>
       <c r="AD19" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.25">
@@ -2806,40 +2806,40 @@
         <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D20" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E20">
-        <v>46203</v>
+        <v>46200</v>
       </c>
       <c r="F20" t="s">
         <v>34</v>
       </c>
       <c r="G20" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="H20" t="s">
-        <v>141</v>
+        <v>40</v>
       </c>
       <c r="I20" t="s">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="J20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K20">
-        <v>13700</v>
+        <v>11030</v>
       </c>
       <c r="L20">
-        <v>49.7</v>
+        <v>44.86</v>
       </c>
       <c r="M20">
-        <v>470.89</v>
+        <v>394.26</v>
       </c>
       <c r="N20" t="s">
-        <v>142</v>
+        <v>40</v>
       </c>
       <c r="O20" t="s">
         <v>40</v>
@@ -2851,13 +2851,13 @@
         <v>1</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="T20" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="U20" t="s">
         <v>44</v>
@@ -2887,7 +2887,7 @@
         <v>52</v>
       </c>
       <c r="AD20" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.25">
@@ -2901,7 +2901,7 @@
         <v>143</v>
       </c>
       <c r="D21" t="s">
-        <v>144</v>
+        <v>40</v>
       </c>
       <c r="E21">
         <v>46200</v>
@@ -2910,49 +2910,49 @@
         <v>34</v>
       </c>
       <c r="G21" t="s">
-        <v>40</v>
+        <v>145</v>
       </c>
       <c r="H21" t="s">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="I21" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K21">
-        <v>11030</v>
+        <v>0</v>
       </c>
       <c r="L21">
-        <v>44.86</v>
+        <v>0</v>
       </c>
       <c r="M21">
-        <v>394.26</v>
+        <v>0</v>
       </c>
       <c r="N21" t="s">
         <v>40</v>
       </c>
       <c r="O21" t="s">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="P21" t="s">
         <v>41</v>
       </c>
       <c r="Q21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
         <v>42</v>
       </c>
       <c r="T21" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="U21" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="V21" t="s">
         <v>45</v>
@@ -2967,7 +2967,7 @@
         <v>48</v>
       </c>
       <c r="Z21" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="AA21" t="s">
         <v>50</v>
@@ -3002,10 +3002,10 @@
         <v>34</v>
       </c>
       <c r="G22" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H22" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I22" t="s">
         <v>48</v>
@@ -3041,7 +3041,7 @@
         <v>42</v>
       </c>
       <c r="T22" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="U22" t="s">
         <v>83</v>
@@ -3082,10 +3082,10 @@
         <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="D23" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="E23">
         <v>46200</v>
@@ -3094,10 +3094,10 @@
         <v>34</v>
       </c>
       <c r="G23" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H23" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I23" t="s">
         <v>48</v>
@@ -3106,13 +3106,13 @@
         <v>38</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>2340</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>69.849999999999994</v>
       </c>
       <c r="M23">
-        <v>0</v>
+        <v>95.21</v>
       </c>
       <c r="N23" t="s">
         <v>40</v>
@@ -3124,19 +3124,19 @@
         <v>41</v>
       </c>
       <c r="Q23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="T23" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="U23" t="s">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="V23" t="s">
         <v>45</v>
@@ -3151,7 +3151,7 @@
         <v>48</v>
       </c>
       <c r="Z23" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="AA23" t="s">
         <v>50</v>
@@ -3163,7 +3163,7 @@
         <v>52</v>
       </c>
       <c r="AD23" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.25">
@@ -3174,10 +3174,10 @@
         <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>123</v>
       </c>
       <c r="D24" t="s">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="E24">
         <v>46200</v>
@@ -3198,13 +3198,13 @@
         <v>40</v>
       </c>
       <c r="K24">
-        <v>2340</v>
+        <v>2390</v>
       </c>
       <c r="L24">
-        <v>69.849999999999994</v>
+        <v>45.39</v>
       </c>
       <c r="M24">
-        <v>95.21</v>
+        <v>78.92</v>
       </c>
       <c r="N24" t="s">
         <v>40</v>
@@ -3266,7 +3266,7 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>123</v>
       </c>
       <c r="D25" t="s">
         <v>40</v>
@@ -3278,10 +3278,10 @@
         <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H25" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I25" t="s">
         <v>48</v>
@@ -3358,43 +3358,43 @@
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="E26">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="F26" t="s">
         <v>34</v>
       </c>
       <c r="G26" t="s">
-        <v>40</v>
+        <v>155</v>
       </c>
       <c r="H26" t="s">
-        <v>40</v>
+        <v>156</v>
       </c>
       <c r="I26" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K26">
-        <v>2390</v>
+        <v>13410</v>
       </c>
       <c r="L26">
-        <v>45.39</v>
+        <v>46.3</v>
       </c>
       <c r="M26">
-        <v>78.92</v>
+        <v>446.64</v>
       </c>
       <c r="N26" t="s">
         <v>40</v>
       </c>
       <c r="O26" t="s">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="P26" t="s">
         <v>41</v>
@@ -3406,10 +3406,10 @@
         <v>1</v>
       </c>
       <c r="S26" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="T26" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="U26" t="s">
         <v>44</v>
@@ -3439,7 +3439,7 @@
         <v>52</v>
       </c>
       <c r="AD26" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.25">
@@ -3450,22 +3450,22 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="D27" t="s">
-        <v>40</v>
+        <v>158</v>
       </c>
       <c r="E27">
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="F27" t="s">
         <v>34</v>
       </c>
       <c r="G27" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="H27" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="I27" t="s">
         <v>48</v>
@@ -3474,13 +3474,13 @@
         <v>38</v>
       </c>
       <c r="K27">
-        <v>0</v>
+        <v>13500</v>
       </c>
       <c r="L27">
-        <v>0</v>
+        <v>35.4</v>
       </c>
       <c r="M27">
-        <v>0</v>
+        <v>403.52</v>
       </c>
       <c r="N27" t="s">
         <v>40</v>
@@ -3492,19 +3492,19 @@
         <v>41</v>
       </c>
       <c r="Q27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" t="s">
-        <v>59</v>
+        <v>161</v>
       </c>
       <c r="T27" t="s">
         <v>43</v>
       </c>
       <c r="U27" t="s">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="V27" t="s">
         <v>45</v>
@@ -3519,7 +3519,7 @@
         <v>48</v>
       </c>
       <c r="Z27" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="AA27" t="s">
         <v>50</v>
@@ -3531,7 +3531,7 @@
         <v>52</v>
       </c>
       <c r="AD27" t="s">
-        <v>60</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">
@@ -3542,22 +3542,22 @@
         <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="D28" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E28">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="F28" t="s">
         <v>34</v>
       </c>
       <c r="G28" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="H28" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="I28" t="s">
         <v>48</v>
@@ -3566,13 +3566,13 @@
         <v>38</v>
       </c>
       <c r="K28">
-        <v>13410</v>
+        <v>13450</v>
       </c>
       <c r="L28">
-        <v>46.3</v>
+        <v>32.17</v>
       </c>
       <c r="M28">
-        <v>446.64</v>
+        <v>388.41</v>
       </c>
       <c r="N28" t="s">
         <v>40</v>
@@ -3590,7 +3590,7 @@
         <v>1</v>
       </c>
       <c r="S28" t="s">
-        <v>42</v>
+        <v>167</v>
       </c>
       <c r="T28" t="s">
         <v>43</v>
@@ -3623,7 +3623,7 @@
         <v>52</v>
       </c>
       <c r="AD28" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.25">
@@ -3634,22 +3634,22 @@
         <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D29" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="E29">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="F29" t="s">
         <v>34</v>
       </c>
       <c r="G29" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="H29" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="I29" t="s">
         <v>48</v>
@@ -3658,13 +3658,13 @@
         <v>38</v>
       </c>
       <c r="K29">
-        <v>13500</v>
+        <v>13120.01</v>
       </c>
       <c r="L29">
-        <v>35.4</v>
+        <v>20.58</v>
       </c>
       <c r="M29">
-        <v>403.52</v>
+        <v>331.23</v>
       </c>
       <c r="N29" t="s">
         <v>40</v>
@@ -3682,7 +3682,7 @@
         <v>1</v>
       </c>
       <c r="S29" t="s">
-        <v>161</v>
+        <v>59</v>
       </c>
       <c r="T29" t="s">
         <v>43</v>
@@ -3715,7 +3715,7 @@
         <v>52</v>
       </c>
       <c r="AD29" t="s">
-        <v>162</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.25">
@@ -3726,10 +3726,10 @@
         <v>31</v>
       </c>
       <c r="C30" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="E30">
         <v>46203</v>
@@ -3738,10 +3738,10 @@
         <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="I30" t="s">
         <v>48</v>
@@ -3750,13 +3750,13 @@
         <v>38</v>
       </c>
       <c r="K30">
-        <v>13450</v>
+        <v>13510</v>
       </c>
       <c r="L30">
-        <v>32.17</v>
+        <v>19.95</v>
       </c>
       <c r="M30">
-        <v>388.41</v>
+        <v>338.41</v>
       </c>
       <c r="N30" t="s">
         <v>40</v>
@@ -3774,7 +3774,7 @@
         <v>1</v>
       </c>
       <c r="S30" t="s">
-        <v>167</v>
+        <v>42</v>
       </c>
       <c r="T30" t="s">
         <v>43</v>
@@ -3807,7 +3807,7 @@
         <v>52</v>
       </c>
       <c r="AD30" t="s">
-        <v>168</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
@@ -3818,43 +3818,43 @@
         <v>31</v>
       </c>
       <c r="C31" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="D31" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="E31">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="F31" t="s">
         <v>34</v>
       </c>
       <c r="G31" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="H31" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="I31" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
       <c r="J31" t="s">
         <v>38</v>
       </c>
       <c r="K31">
-        <v>13120.01</v>
+        <v>13870</v>
       </c>
       <c r="L31">
-        <v>20.58</v>
+        <v>66.61</v>
       </c>
       <c r="M31">
-        <v>331.23</v>
+        <v>550.24</v>
       </c>
       <c r="N31" t="s">
-        <v>40</v>
+        <v>181</v>
       </c>
       <c r="O31" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
       <c r="P31" t="s">
         <v>41</v>
@@ -3910,43 +3910,43 @@
         <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D32" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="E32">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="F32" t="s">
         <v>34</v>
       </c>
       <c r="G32" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="H32" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="I32" t="s">
-        <v>48</v>
+        <v>186</v>
       </c>
       <c r="J32" t="s">
         <v>38</v>
       </c>
       <c r="K32">
-        <v>13510</v>
+        <v>13560</v>
       </c>
       <c r="L32">
-        <v>19.95</v>
+        <v>131.69999999999999</v>
       </c>
       <c r="M32">
-        <v>338.41</v>
+        <v>814.52</v>
       </c>
       <c r="N32" t="s">
-        <v>40</v>
+        <v>187</v>
       </c>
       <c r="O32" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
       <c r="P32" t="s">
         <v>41</v>
@@ -3958,7 +3958,7 @@
         <v>1</v>
       </c>
       <c r="S32" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="T32" t="s">
         <v>43</v>
@@ -3991,7 +3991,7 @@
         <v>52</v>
       </c>
       <c r="AD32" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.25">
@@ -4002,10 +4002,10 @@
         <v>31</v>
       </c>
       <c r="C33" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="D33" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="E33">
         <v>46204</v>
@@ -4014,28 +4014,28 @@
         <v>34</v>
       </c>
       <c r="G33" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="H33" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="I33" t="s">
-        <v>105</v>
+        <v>48</v>
       </c>
       <c r="J33" t="s">
         <v>38</v>
       </c>
       <c r="K33">
-        <v>13870</v>
+        <v>12110</v>
       </c>
       <c r="L33">
-        <v>66.61</v>
+        <v>46.5</v>
       </c>
       <c r="M33">
-        <v>550.24</v>
+        <v>404.1</v>
       </c>
       <c r="N33" t="s">
-        <v>181</v>
+        <v>40</v>
       </c>
       <c r="O33" t="s">
         <v>40</v>
@@ -4094,40 +4094,40 @@
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="D34" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="E34">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="F34" t="s">
         <v>34</v>
       </c>
       <c r="G34" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="H34" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="I34" t="s">
-        <v>186</v>
+        <v>88</v>
       </c>
       <c r="J34" t="s">
         <v>38</v>
       </c>
       <c r="K34">
-        <v>13560</v>
+        <v>13570</v>
       </c>
       <c r="L34">
-        <v>131.69999999999999</v>
+        <v>73.61</v>
       </c>
       <c r="M34">
-        <v>814.52</v>
+        <v>568.1</v>
       </c>
       <c r="N34" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="O34" t="s">
         <v>40</v>
@@ -4142,7 +4142,7 @@
         <v>1</v>
       </c>
       <c r="S34" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="T34" t="s">
         <v>43</v>
@@ -4175,7 +4175,7 @@
         <v>52</v>
       </c>
       <c r="AD34" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.25">
@@ -4186,10 +4186,10 @@
         <v>31</v>
       </c>
       <c r="C35" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="D35" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="E35">
         <v>46204</v>
@@ -4198,28 +4198,28 @@
         <v>34</v>
       </c>
       <c r="G35" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="H35" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="I35" t="s">
-        <v>48</v>
+        <v>186</v>
       </c>
       <c r="J35" t="s">
         <v>38</v>
       </c>
       <c r="K35">
-        <v>12110</v>
+        <v>13860</v>
       </c>
       <c r="L35">
-        <v>46.5</v>
+        <v>131.69999999999999</v>
       </c>
       <c r="M35">
-        <v>404.1</v>
+        <v>832.54</v>
       </c>
       <c r="N35" t="s">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="O35" t="s">
         <v>40</v>
@@ -4234,7 +4234,7 @@
         <v>1</v>
       </c>
       <c r="S35" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="T35" t="s">
         <v>43</v>
@@ -4267,7 +4267,7 @@
         <v>52</v>
       </c>
       <c r="AD35" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.25">
@@ -4278,10 +4278,10 @@
         <v>31</v>
       </c>
       <c r="C36" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="D36" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="E36">
         <v>46205</v>
@@ -4290,28 +4290,28 @@
         <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H36" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="I36" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="J36" t="s">
         <v>38</v>
       </c>
       <c r="K36">
-        <v>13570</v>
+        <v>12820</v>
       </c>
       <c r="L36">
-        <v>73.61</v>
+        <v>58.72</v>
       </c>
       <c r="M36">
-        <v>568.1</v>
+        <v>476.88</v>
       </c>
       <c r="N36" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="O36" t="s">
         <v>40</v>
@@ -4326,7 +4326,7 @@
         <v>1</v>
       </c>
       <c r="S36" t="s">
-        <v>42</v>
+        <v>206</v>
       </c>
       <c r="T36" t="s">
         <v>43</v>
@@ -4359,7 +4359,7 @@
         <v>52</v>
       </c>
       <c r="AD36" t="s">
-        <v>53</v>
+        <v>207</v>
       </c>
     </row>
     <row r="37" spans="1:30" x14ac:dyDescent="0.25">
@@ -4370,40 +4370,40 @@
         <v>31</v>
       </c>
       <c r="C37" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="D37" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="E37">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="F37" t="s">
         <v>34</v>
       </c>
       <c r="G37" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="H37" t="s">
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="I37" t="s">
-        <v>186</v>
+        <v>105</v>
       </c>
       <c r="J37" t="s">
         <v>38</v>
       </c>
       <c r="K37">
-        <v>13860</v>
+        <v>13660</v>
       </c>
       <c r="L37">
-        <v>131.69999999999999</v>
+        <v>47.75</v>
       </c>
       <c r="M37">
-        <v>832.54</v>
+        <v>461.17</v>
       </c>
       <c r="N37" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="O37" t="s">
         <v>40</v>
@@ -4418,7 +4418,7 @@
         <v>1</v>
       </c>
       <c r="S37" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="T37" t="s">
         <v>43</v>
@@ -4451,190 +4451,6 @@
         <v>52</v>
       </c>
       <c r="AD37" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" t="s">
-        <v>31</v>
-      </c>
-      <c r="C38" t="s">
-        <v>201</v>
-      </c>
-      <c r="D38" t="s">
-        <v>202</v>
-      </c>
-      <c r="E38">
-        <v>46205</v>
-      </c>
-      <c r="F38" t="s">
-        <v>34</v>
-      </c>
-      <c r="G38" t="s">
-        <v>203</v>
-      </c>
-      <c r="H38" t="s">
-        <v>204</v>
-      </c>
-      <c r="I38" t="s">
-        <v>65</v>
-      </c>
-      <c r="J38" t="s">
-        <v>38</v>
-      </c>
-      <c r="K38">
-        <v>12820</v>
-      </c>
-      <c r="L38">
-        <v>58.72</v>
-      </c>
-      <c r="M38">
-        <v>476.88</v>
-      </c>
-      <c r="N38" t="s">
-        <v>205</v>
-      </c>
-      <c r="O38" t="s">
-        <v>40</v>
-      </c>
-      <c r="P38" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q38">
-        <v>1</v>
-      </c>
-      <c r="R38">
-        <v>1</v>
-      </c>
-      <c r="S38" t="s">
-        <v>206</v>
-      </c>
-      <c r="T38" t="s">
-        <v>43</v>
-      </c>
-      <c r="U38" t="s">
-        <v>44</v>
-      </c>
-      <c r="V38" t="s">
-        <v>45</v>
-      </c>
-      <c r="W38" t="s">
-        <v>46</v>
-      </c>
-      <c r="X38" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y38" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z38" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA38" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB38" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC38" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD38" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" t="s">
-        <v>31</v>
-      </c>
-      <c r="C39" t="s">
-        <v>208</v>
-      </c>
-      <c r="D39" t="s">
-        <v>209</v>
-      </c>
-      <c r="E39">
-        <v>46205</v>
-      </c>
-      <c r="F39" t="s">
-        <v>34</v>
-      </c>
-      <c r="G39" t="s">
-        <v>210</v>
-      </c>
-      <c r="H39" t="s">
-        <v>211</v>
-      </c>
-      <c r="I39" t="s">
-        <v>105</v>
-      </c>
-      <c r="J39" t="s">
-        <v>38</v>
-      </c>
-      <c r="K39">
-        <v>13660</v>
-      </c>
-      <c r="L39">
-        <v>47.75</v>
-      </c>
-      <c r="M39">
-        <v>461.17</v>
-      </c>
-      <c r="N39" t="s">
-        <v>212</v>
-      </c>
-      <c r="O39" t="s">
-        <v>40</v>
-      </c>
-      <c r="P39" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q39">
-        <v>1</v>
-      </c>
-      <c r="R39">
-        <v>1</v>
-      </c>
-      <c r="S39" t="s">
-        <v>59</v>
-      </c>
-      <c r="T39" t="s">
-        <v>43</v>
-      </c>
-      <c r="U39" t="s">
-        <v>44</v>
-      </c>
-      <c r="V39" t="s">
-        <v>45</v>
-      </c>
-      <c r="W39" t="s">
-        <v>46</v>
-      </c>
-      <c r="X39" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y39" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z39" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA39" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB39" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC39" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD39" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>